<commit_message>
feat: add execute_python tool + briefing mode + bug fixes
- executor.py: JSON parse fix for LLM tool call arguments (string -> dict)
- executor.py: execute_python moved before script_tools_enabled guard (inline calc always allowed)
- tool_schemas.py: add execute_python, ingest_battlefield_data, generate_briefing, recommend_coa schemas
- battlefield.py: new module - CSV/JSON ingestion + BLUF+SALUTE briefing prompts
- main.py: add /api/briefing endpoint + DEFENSE_LLM_SCRIPT_TOOLS_ENABLED env var + mock adapter fix
- web QueryPage.jsx: briefing mode UI + calculation examples + AgentTracePanel
- web IndexPage.jsx: PDF upload support

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/0.FilesUpdate.xlsx
+++ b/0.FilesUpdate.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -578,6 +578,108 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-20 16:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>src/defense_llm/agent/battlefield.py</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DataIngester(CSV/JSON 파싱) + BriefingFormatter 신규 모듈</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-20 16:30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>src/defense_llm/agent/tool_schemas.py</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>execute_python / ingest_battlefield_data / generate_briefing / recommend_coa tool 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-20 16:30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>src/defense_llm/agent/executor.py</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>situation_data 상태 관리, 4개 tool dispatcher 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-03-20 16:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>src/defense_llm/api/main.py</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>security_enabled 버그 수정, /api/briefing 엔드포인트 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-03-20 16:30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>web/src/pages/QueryPage.jsx</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Briefing 모드 UI 추가 (CSV/JSON 입력, COA 표시), 계산 예시 쿼리 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03-20 16:30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>web/src/pages/IndexPage.jsx</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PDF 파일 업로드 지원 추가</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>